<commit_message>
feat: deliver Dayu Tiangong Phase 3 and 4
</commit_message>
<xml_diff>
--- a/docs/templates/phase2_cross_sections_template.xlsx
+++ b/docs/templates/phase2_cross_sections_template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导入数据" sheetId="1" r:id="Rec6e64b6112948cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R64fa1fe21ac245fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导入数据" sheetId="1" r:id="R8fa719cae05f4fad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rc17a977157b64814"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -190,7 +190,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="44">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -249,6 +249,33 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1047,7 +1074,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d105494b8b4458c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2ba78169b8d4c3a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1140,34 +1167,40 @@
         <x:v>0.035</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="26" t="str">
+    <x:row r="9" ht="25" customHeight="1">
+      <x:c r="A9" s="35" t="str">
         <x:v>使用说明：
 1. 导入时由页面选择数据版本，模板内不填写版本 ID。
 2. 第一行字段名不可修改；请删除示例行后填写正式数据。
-3. 坐标统一使用 WGS 84（EPSG:4326）。
+3. 坐标统一使用 CGCS2000（EPSG:4490），坐标顺序为 [经度,纬度]。
 4. 任一行错误时整批不写入，错误会定位到具体行号。</x:v>
       </x:c>
-      <x:c r="B9" s="27"/>
-      <x:c r="C9" s="27"/>
-      <x:c r="D9" s="28"/>
+      <x:c r="B9" s="36"/>
+      <x:c r="C9" s="36"/>
+      <x:c r="D9" s="37"/>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="29"/>
-      <x:c r="B10" s="30"/>
-      <x:c r="C10" s="30"/>
-      <x:c r="D10" s="31"/>
+    <x:row r="10" ht="25" customHeight="1">
+      <x:c r="A10" s="38"/>
+      <x:c r="B10" s="39"/>
+      <x:c r="C10" s="39"/>
+      <x:c r="D10" s="40"/>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="32"/>
-      <x:c r="B11" s="33"/>
-      <x:c r="C11" s="33"/>
-      <x:c r="D11" s="34"/>
+    <x:row r="11" ht="25" customHeight="1">
+      <x:c r="A11" s="38"/>
+      <x:c r="B11" s="39"/>
+      <x:c r="C11" s="39"/>
+      <x:c r="D11" s="40"/>
+    </x:row>
+    <x:row r="12" ht="25" customHeight="1">
+      <x:c r="A12" s="41"/>
+      <x:c r="B12" s="42"/>
+      <x:c r="C12" s="42"/>
+      <x:c r="D12" s="43"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>
-    <x:mergeCell ref="A9:D11"/>
+    <x:mergeCell ref="A9:D12"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>